<commit_message>
Mayo highnoise_v2: 150-200 eval/train setup + per-patient configs
config/mayo_ct_denoise.json + new per-patient configs (L291, L310) with datasets.train slice_range=[150,200]; data/mayo_ct_dataset.py slice-window logic (end=min(num_slices,200)); eval_mayo.py (EVAL_SLICE_START/END=150/200, crop_eval_slices); inference_mayo.py; model diffusion.py; per-patient result xlsx. Excludes __pycache__, Untitled-1.ipynb, and experiments/ checkpoints.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mayo_ddm2_results.xlsx
+++ b/mayo_ddm2_results.xlsx
@@ -508,7 +508,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>L291</t>
+          <t>L192</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -517,43 +517,43 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>19.61916471702087</v>
+        <v>18.09102950231616</v>
       </c>
       <c r="E2" t="n">
-        <v>14.06383506198891</v>
+        <v>13.46782899427272</v>
       </c>
       <c r="F2" t="n">
-        <v>14.32115893149725</v>
+        <v>13.16955323655913</v>
       </c>
       <c r="G2" t="n">
-        <v>17.46457110767492</v>
+        <v>14.06363364646359</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6987833793634104</v>
+        <v>0.6983741103546943</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7369427260308268</v>
+        <v>0.7300221312738004</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7380197776386977</v>
+        <v>0.7229662521224046</v>
       </c>
       <c r="K2" t="n">
-        <v>0.6339152061558513</v>
+        <v>0.6871998440635133</v>
       </c>
       <c r="L2" t="n">
-        <v>0.09804286226630211</v>
+        <v>0.08503647893667221</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1235505582392216</v>
+        <v>0.08850082486867905</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1290383235365152</v>
+        <v>0.08347253888845443</v>
       </c>
       <c r="O2" t="n">
-        <v>0.2420408920943737</v>
+        <v>0.09533699408173561</v>
       </c>
     </row>
   </sheetData>

</xml_diff>